<commit_message>
feat: handler de document-generation confirmado por el equipo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lambdas.xlsx
+++ b/lambdas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miguel.fernandez\MEFS-DELOSI\repo_gitlab\ventasCorp-infrastructure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{216D848B-A39A-4E54-AF25-83976D45B4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B538ED25-F27E-4CE2-9CC0-FB37F4CB2A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BEF15F6B-496F-4DCF-8342-CC49EC0D1F13}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3976C1CF-DEC9-4EF3-94A9-D9453447DCA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Lambdas de API" sheetId="1" r:id="rId1"/>
@@ -316,10 +316,10 @@
     <t>document-generation</t>
   </si>
   <si>
-    <t>Delosi.DocumentGeneration</t>
-  </si>
-  <si>
-    <t>Delosi.DocumentGeneration.Functions.DocumentGenerationFunction</t>
+    <t>Delosi.Alfie.Document.Generation.Functions</t>
+  </si>
+  <si>
+    <t>Delosi.Alfie.Document.Generation.Functions.DocumentGenerationFunction</t>
   </si>
   <si>
     <t>delosi-ventascorp-{env}/document-generation-db
@@ -737,7 +737,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8356BE69-3C91-4473-8941-1D6C279ABD9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EA43BA-A7DF-4A81-8A38-C67E778031EE}">
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1001,7 +1001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D23CA69-A2DE-471E-A574-5762640FE7D4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CB9E422-1B9C-4F26-9BFE-AC8A5D361529}">
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1144,7 +1144,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37896E16-34CB-4FC9-A0D5-51CA2038DEB2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C48333A4-5565-4E55-9224-675232AB67ED}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>